<commit_message>
Functional "Engine" class.  Entity factories return pointer instead of instance. Toggleable print on scene EOL. Benchmark file generation.
</commit_message>
<xml_diff>
--- a/Randor_simplu/Documentation/Performance Review.xlsx
+++ b/Randor_simplu/Documentation/Performance Review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZentriX\source\repos\Randor_simplu\Randor_simplu\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94687FAA-C0A6-4296-B03B-79F6A0D508A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F156A19-15D8-4F11-9046-D5DF879DE314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="91">
   <si>
     <t>Benchmark</t>
   </si>
@@ -193,13 +193,121 @@
   </si>
   <si>
     <t>Throughput saturation</t>
+  </si>
+  <si>
+    <t>Entities</t>
+  </si>
+  <si>
+    <t>Physics</t>
+  </si>
+  <si>
+    <t>Frame</t>
+  </si>
+  <si>
+    <t>Physics Share</t>
+  </si>
+  <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>11.18 ms</t>
+  </si>
+  <si>
+    <t>3k</t>
+  </si>
+  <si>
+    <t>34.29 ms</t>
+  </si>
+  <si>
+    <t>34.28 ms</t>
+  </si>
+  <si>
+    <t>5k</t>
+  </si>
+  <si>
+    <t>54.49 ms</t>
+  </si>
+  <si>
+    <t>54.46 ms</t>
+  </si>
+  <si>
+    <t>7k</t>
+  </si>
+  <si>
+    <t>76.45 ms</t>
+  </si>
+  <si>
+    <t>76.40 ms</t>
+  </si>
+  <si>
+    <t>9k</t>
+  </si>
+  <si>
+    <t>107.51 ms</t>
+  </si>
+  <si>
+    <t>107.43 ms</t>
+  </si>
+  <si>
+    <t>11k</t>
+  </si>
+  <si>
+    <t>119.48 ms</t>
+  </si>
+  <si>
+    <t>119.38 ms</t>
+  </si>
+  <si>
+    <t>21k</t>
+  </si>
+  <si>
+    <t>229.29 ms</t>
+  </si>
+  <si>
+    <t>228.91 ms</t>
+  </si>
+  <si>
+    <t>31k</t>
+  </si>
+  <si>
+    <t>357.23 ms</t>
+  </si>
+  <si>
+    <t>356.35 ms</t>
+  </si>
+  <si>
+    <t>41k</t>
+  </si>
+  <si>
+    <t>467.19 ms</t>
+  </si>
+  <si>
+    <t>465.61 ms</t>
+  </si>
+  <si>
+    <t>51k</t>
+  </si>
+  <si>
+    <t>579.82 ms</t>
+  </si>
+  <si>
+    <t>577.54 ms</t>
+  </si>
+  <si>
+    <t>81k</t>
+  </si>
+  <si>
+    <t>1030.21 ms</t>
+  </si>
+  <si>
+    <t>1018.19 ms</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -246,6 +354,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF760006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -337,7 +453,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -383,6 +499,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -393,6 +527,22 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -428,22 +578,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </right>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -464,7 +598,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{91A1803D-FC57-4E91-B209-8D74327FF863}" name="Table5" displayName="Table5" ref="A1:F12" totalsRowShown="0" headerRowDxfId="0" tableBorderDxfId="1" headerRowCellStyle="Heading 4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{91A1803D-FC57-4E91-B209-8D74327FF863}" name="Table5" displayName="Table5" ref="A1:F12" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0" headerRowCellStyle="Heading 4">
   <autoFilter ref="A1:F12" xr:uid="{91A1803D-FC57-4E91-B209-8D74327FF863}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2B1AA87A-8AC2-4210-823C-3BAA4BB9EBD7}" name="Benchmark"/>
@@ -741,7 +875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -750,11 +884,12 @@
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="36.42578125" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="8" max="8" width="21.7109375" customWidth="1"/>
-    <col min="9" max="9" width="5.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" style="21" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -773,8 +908,20 @@
       <c r="F1" s="15" t="s">
         <v>50</v>
       </c>
+      <c r="H1" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -793,8 +940,20 @@
       <c r="F2" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="H2" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="I2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="K2" s="18">
+        <v>0.99990000000000001</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -813,8 +972,20 @@
       <c r="F3" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="H3" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" s="18">
+        <v>1.0003</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
@@ -833,8 +1004,20 @@
       <c r="F4" s="6" t="s">
         <v>52</v>
       </c>
+      <c r="H4" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="K4" s="18">
+        <v>1.0004</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
@@ -853,8 +1036,20 @@
       <c r="F5" s="6" t="s">
         <v>52</v>
       </c>
+      <c r="H5" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="K5" s="18">
+        <v>1.0005999999999999</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
@@ -873,8 +1068,20 @@
       <c r="F6" s="6" t="s">
         <v>52</v>
       </c>
+      <c r="H6" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="K6" s="18">
+        <v>1.0006999999999999</v>
+      </c>
     </row>
-    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>27</v>
       </c>
@@ -893,8 +1100,20 @@
       <c r="F7" s="6" t="s">
         <v>52</v>
       </c>
+      <c r="H7" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="18">
+        <v>1.0008999999999999</v>
+      </c>
     </row>
-    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>31</v>
       </c>
@@ -913,8 +1132,20 @@
       <c r="F8" s="6" t="s">
         <v>52</v>
       </c>
+      <c r="H8" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="K8" s="18">
+        <v>1.0017</v>
+      </c>
     </row>
-    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
@@ -933,8 +1164,20 @@
       <c r="F9" s="9" t="s">
         <v>53</v>
       </c>
+      <c r="H9" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="K9" s="18">
+        <v>1.0024999999999999</v>
+      </c>
     </row>
-    <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
@@ -953,8 +1196,20 @@
       <c r="F10" s="9" t="s">
         <v>53</v>
       </c>
+      <c r="H10" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="J10" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="K10" s="18">
+        <v>1.0034000000000001</v>
+      </c>
     </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>42</v>
       </c>
@@ -973,8 +1228,20 @@
       <c r="F11" s="12" t="s">
         <v>54</v>
       </c>
+      <c r="H11" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="18">
+        <v>1.0039</v>
+      </c>
     </row>
-    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>46</v>
       </c>
@@ -992,6 +1259,18 @@
       </c>
       <c r="F12" s="12" t="s">
         <v>54</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="J12" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="K12" s="18">
+        <v>1.0118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expanded FrameStat for rendering stages. Compile-time "FRAME_PROFILER" switch in Macros.h Moved most such switches there.
</commit_message>
<xml_diff>
--- a/Randor_simplu/Documentation/Performance Review.xlsx
+++ b/Randor_simplu/Documentation/Performance Review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZentriX\source\repos\Randor_simplu\Randor_simplu\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F156A19-15D8-4F11-9046-D5DF879DE314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36ED5C35-EFEF-4F3E-A119-7073FA1AF0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="90">
   <si>
     <t>Benchmark</t>
   </si>
@@ -198,109 +198,106 @@
     <t>Entities</t>
   </si>
   <si>
-    <t>Physics</t>
-  </si>
-  <si>
-    <t>Frame</t>
-  </si>
-  <si>
-    <t>Physics Share</t>
-  </si>
-  <si>
-    <t>1k</t>
-  </si>
-  <si>
-    <t>11.18 ms</t>
-  </si>
-  <si>
-    <t>3k</t>
-  </si>
-  <si>
-    <t>34.29 ms</t>
-  </si>
-  <si>
-    <t>34.28 ms</t>
-  </si>
-  <si>
-    <t>5k</t>
-  </si>
-  <si>
-    <t>54.49 ms</t>
-  </si>
-  <si>
-    <t>54.46 ms</t>
-  </si>
-  <si>
-    <t>7k</t>
-  </si>
-  <si>
-    <t>76.45 ms</t>
-  </si>
-  <si>
-    <t>76.40 ms</t>
-  </si>
-  <si>
-    <t>9k</t>
-  </si>
-  <si>
-    <t>107.51 ms</t>
-  </si>
-  <si>
-    <t>107.43 ms</t>
-  </si>
-  <si>
-    <t>11k</t>
-  </si>
-  <si>
-    <t>119.48 ms</t>
-  </si>
-  <si>
-    <t>119.38 ms</t>
-  </si>
-  <si>
-    <t>21k</t>
-  </si>
-  <si>
-    <t>229.29 ms</t>
-  </si>
-  <si>
-    <t>228.91 ms</t>
-  </si>
-  <si>
-    <t>31k</t>
-  </si>
-  <si>
-    <t>357.23 ms</t>
-  </si>
-  <si>
-    <t>356.35 ms</t>
-  </si>
-  <si>
-    <t>41k</t>
-  </si>
-  <si>
-    <t>467.19 ms</t>
-  </si>
-  <si>
-    <t>465.61 ms</t>
-  </si>
-  <si>
-    <t>51k</t>
-  </si>
-  <si>
-    <t>579.82 ms</t>
-  </si>
-  <si>
-    <t>577.54 ms</t>
-  </si>
-  <si>
-    <t>81k</t>
-  </si>
-  <si>
-    <t>1030.21 ms</t>
-  </si>
-  <si>
-    <t>1018.19 ms</t>
+    <t>Physics (ms)</t>
+  </si>
+  <si>
+    <t>Frame (ms)</t>
+  </si>
+  <si>
+    <t>FPS</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>169 MB</t>
+  </si>
+  <si>
+    <t>208 MB</t>
+  </si>
+  <si>
+    <t>253 MB</t>
+  </si>
+  <si>
+    <t>412 MB</t>
+  </si>
+  <si>
+    <t>596 MB</t>
+  </si>
+  <si>
+    <t>804 MB</t>
+  </si>
+  <si>
+    <t>1036 MB</t>
+  </si>
+  <si>
+    <t>1432 MB</t>
+  </si>
+  <si>
+    <t>DEBUG</t>
+  </si>
+  <si>
+    <t>Approx FPS</t>
+  </si>
+  <si>
+    <t>Relative to Debug</t>
+  </si>
+  <si>
+    <t>~12.4</t>
+  </si>
+  <si>
+    <t>~80</t>
+  </si>
+  <si>
+    <t>~6× faster</t>
+  </si>
+  <si>
+    <t>~15.3</t>
+  </si>
+  <si>
+    <t>~65</t>
+  </si>
+  <si>
+    <t>~6.5× faster</t>
+  </si>
+  <si>
+    <t>~18–19</t>
+  </si>
+  <si>
+    <t>~53</t>
+  </si>
+  <si>
+    <t>~36–38</t>
+  </si>
+  <si>
+    <t>~27</t>
+  </si>
+  <si>
+    <t>~58–60</t>
+  </si>
+  <si>
+    <t>~17</t>
+  </si>
+  <si>
+    <t>~74–78</t>
+  </si>
+  <si>
+    <t>~13</t>
+  </si>
+  <si>
+    <t>~92–94</t>
+  </si>
+  <si>
+    <t>~11</t>
+  </si>
+  <si>
+    <t>~124–126</t>
+  </si>
+  <si>
+    <t>~8</t>
+  </si>
+  <si>
+    <t>RELEASE</t>
   </si>
 </sst>
 </file>
@@ -367,7 +364,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -405,6 +402,18 @@
       <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -453,7 +462,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -509,13 +518,21 @@
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -875,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -885,11 +902,10 @@
     <col min="5" max="5" width="36.42578125" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" style="21" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -908,20 +924,20 @@
       <c r="F1" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>58</v>
-      </c>
+      <c r="H1" s="22"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
-    <row r="2" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -940,20 +956,32 @@
       <c r="F2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="I2" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="J2" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="K2" s="18">
-        <v>0.99990000000000001</v>
+      <c r="I2" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="M2" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="N2" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="O2" s="17" t="s">
+        <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -972,20 +1000,32 @@
       <c r="F3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H3" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="I3" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="K3" s="18">
-        <v>1.0003</v>
+      <c r="H3" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" s="20">
+        <v>7000</v>
+      </c>
+      <c r="J3" s="16">
+        <v>75.72</v>
+      </c>
+      <c r="K3" s="16">
+        <v>75.73</v>
+      </c>
+      <c r="L3" s="16">
+        <v>13.21</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
@@ -1004,20 +1044,32 @@
       <c r="F4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="K4" s="18">
-        <v>1.0004</v>
+      <c r="H4" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="20">
+        <v>9000</v>
+      </c>
+      <c r="J4" s="16">
+        <v>98.78</v>
+      </c>
+      <c r="K4" s="16">
+        <v>98.81</v>
+      </c>
+      <c r="L4" s="16">
+        <v>10.119999999999999</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="O4" s="16" t="s">
+        <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
@@ -1036,20 +1088,32 @@
       <c r="F5" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="I5" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="K5" s="18">
-        <v>1.0005999999999999</v>
+      <c r="H5" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="20">
+        <v>11000</v>
+      </c>
+      <c r="J5" s="16">
+        <v>119.74</v>
+      </c>
+      <c r="K5" s="16">
+        <v>119.78</v>
+      </c>
+      <c r="L5" s="16">
+        <v>8.35</v>
+      </c>
+      <c r="M5" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="N5" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="O5" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
@@ -1068,20 +1132,32 @@
       <c r="F6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="I6" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="K6" s="18">
-        <v>1.0006999999999999</v>
+      <c r="H6" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="20">
+        <v>21000</v>
+      </c>
+      <c r="J6" s="16">
+        <v>228.17</v>
+      </c>
+      <c r="K6" s="16">
+        <v>228.31</v>
+      </c>
+      <c r="L6" s="16">
+        <v>4.38</v>
+      </c>
+      <c r="M6" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="N6" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>27</v>
       </c>
@@ -1100,20 +1176,32 @@
       <c r="F7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="20">
+        <v>31000</v>
+      </c>
+      <c r="J7" s="16">
+        <v>353.27</v>
+      </c>
+      <c r="K7" s="16">
+        <v>353.58</v>
+      </c>
+      <c r="L7" s="16">
+        <v>2.83</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="O7" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="I7" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="J7" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="K7" s="18">
-        <v>1.0008999999999999</v>
-      </c>
     </row>
-    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>31</v>
       </c>
@@ -1132,20 +1220,32 @@
       <c r="F8" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="I8" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="J8" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="K8" s="18">
-        <v>1.0017</v>
+      <c r="H8" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="I8" s="20">
+        <v>41000</v>
+      </c>
+      <c r="J8" s="16">
+        <v>468.18</v>
+      </c>
+      <c r="K8" s="16">
+        <v>468.7</v>
+      </c>
+      <c r="L8" s="16">
+        <v>2.14</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="N8" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="O8" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
@@ -1164,20 +1264,32 @@
       <c r="F9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="H9" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="I9" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="K9" s="18">
-        <v>1.0024999999999999</v>
+      <c r="H9" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="20">
+        <v>51000</v>
+      </c>
+      <c r="J9" s="16">
+        <v>550.78</v>
+      </c>
+      <c r="K9" s="16">
+        <v>551.51</v>
+      </c>
+      <c r="L9" s="16">
+        <v>1.82</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="N9" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="O9" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
@@ -1196,20 +1308,32 @@
       <c r="F10" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="I10" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="J10" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="K10" s="18">
-        <v>1.0034000000000001</v>
+      <c r="H10" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" s="20">
+        <v>71000</v>
+      </c>
+      <c r="J10" s="16">
+        <v>773.35</v>
+      </c>
+      <c r="K10" s="16">
+        <v>774.81</v>
+      </c>
+      <c r="L10" s="16">
+        <v>1.29</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="N10" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="O10" s="16" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>42</v>
       </c>
@@ -1228,20 +1352,12 @@
       <c r="F11" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="H11" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="I11" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="J11" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="K11" s="18">
-        <v>1.0039</v>
-      </c>
+      <c r="I11" s="19"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="18"/>
     </row>
-    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>46</v>
       </c>
@@ -1260,20 +1376,15 @@
       <c r="F12" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="H12" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="I12" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="J12" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="K12" s="18">
-        <v>1.0118</v>
-      </c>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="18"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:O1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>